<commit_message>
Actualizaci├│n de repositorio automatizado con .bat
</commit_message>
<xml_diff>
--- a/Tema 2/ProblemarioTema 2.xlsx
+++ b/Tema 2/ProblemarioTema 2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\varga\Desktop\Metodos Numericos\Repositorio\Tema 2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FC240B9B-CE37-46B9-A726-E2690A9F2E99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF277BC8-0BB3-40F7-BD1F-75A8632C49CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="16305" firstSheet="13" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" firstSheet="13" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Metodo de Newthon" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,6 @@
     <sheet name="Metodo de Regla Falsa4" sheetId="15" r:id="rId15"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>

</xml_diff>